<commit_message>
register work is done
</commit_message>
<xml_diff>
--- a/config/plc_data.xlsx
+++ b/config/plc_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,14 +526,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>192.168.96.58</t>
+          <t>127.0.0.1</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D5" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E5" t="n">
         <v>5</v>
@@ -746,6 +746,27 @@
         <v>100</v>
       </c>
       <c r="E15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PLC15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>192.168.1.100</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>505</v>
+      </c>
+      <c r="D16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
register work is done and removed unwanted files
</commit_message>
<xml_diff>
--- a/config/plc_data.xlsx
+++ b/config/plc_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,10 +470,10 @@
         <v>501</v>
       </c>
       <c r="D2" t="n">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -484,14 +484,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>127.0.0.1</t>
+          <t>192.168.15.1</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>502</v>
       </c>
       <c r="D3" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
@@ -512,7 +512,7 @@
         <v>503</v>
       </c>
       <c r="D4" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E4" t="n">
         <v>5</v>
@@ -545,19 +545,15 @@
           <t>PLC5</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>192.168.10.100</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -566,19 +562,15 @@
           <t>PLC6</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="n">
-        <v>555</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>100</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -587,19 +579,15 @@
           <t>PLC7</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
         <v>100</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -608,19 +596,15 @@
           <t>PLC8</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="E9" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -629,16 +613,12 @@
           <t>PLC9</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="n">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -650,19 +630,15 @@
           <t>PLC10</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
         <v>100</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -671,19 +647,15 @@
           <t>PLC11</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>100</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -692,19 +664,15 @@
           <t>PLC12</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -713,19 +681,15 @@
           <t>PLC13</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>192.168.1.11</t>
-        </is>
-      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>502</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>100</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -734,19 +698,15 @@
           <t>PLC14</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>192.168.1.1</t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>100</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -755,19 +715,100 @@
           <t>PLC15</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>192.168.1.100</t>
-        </is>
-      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>100</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PLC16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PLC17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PLC18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PLC19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PLC20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>